<commit_message>
feat: complete F6 phase (catalogo, presupuestos pipeline, paquetes, branding)
- Catalogo: jerarquia tipo_analisis/metodo con snapshots (F6.3)
- Presupuestos: pipeline de estados + Kanban, dual mode y pricing por linea (F6.2, F6.5)
- Paquetes: armado por grupos + precio base (F6.4)
- Branding PDF RV Laboratorio + config institucional (F6.6)
- Core: login en /, password recovery, edad/sexo pacientes (F6.1)
- Fix: lint no-explicit-any, ADR-08 (auth server a apps/web), cableado modulo Config
</commit_message>
<xml_diff>
--- a/apps/web/public/plantilla-import.xlsx
+++ b/apps/web/public/plantilla-import.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:G3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -415,6 +415,12 @@
       <c r="E1" t="str">
         <v>Valores de Referencia</v>
       </c>
+      <c r="F1" t="str">
+        <v>Tipo de Análisis</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Método</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -432,6 +438,12 @@
       <c r="E2" t="str">
         <v>Leucocitos: 4.5-11.0 x10^3/uL</v>
       </c>
+      <c r="F2" t="str">
+        <v>Hematología</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Impedancia eléctrica</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -449,10 +461,16 @@
       <c r="E3" t="str">
         <v>70 - 100 mg/dL</v>
       </c>
+      <c r="F3" t="str">
+        <v>Química clínica</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Método enzimático (glucosa oxidasa)</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>